<commit_message>
fix: remove empty crossover row/CROSSFL from example (shell, spec, data)
The Week-16 placebo crossover disposition row rendered n=0 in every arm
(no CROSSFL='Y' subjects in the synthetic data) and was already absent
from the inputs shell. Purge it everywhere so the inst shell matches:

- inst annotated shell: drop the "Crossed over from Placebo" table row.
- Both specs: delete the ADSL CROSSFL variable row.
- All ADSL datasets (inputs loose + both ADaM.zip): drop the CROSSFL column.

Annotation/spec/dataset alignment re-verified: no orphans, no >8-char
names, spec == dataset for both file sets.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inputs/adam_spec_APX-DRM-301.xlsx
+++ b/inputs/adam_spec_APX-DRM-301.xlsx
@@ -3589,7 +3589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M82"/>
+  <dimension ref="A1:M81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -6634,12 +6634,12 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>CROSSFL</t>
+          <t>STRAT1</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Crossover Flag</t>
+          <t>Stratification Factor 1</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
@@ -6648,7 +6648,7 @@
         </is>
       </c>
       <c r="E54" s="5" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
@@ -6660,20 +6660,16 @@
           <t>Perm</t>
         </is>
       </c>
-      <c r="H54" s="5" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
+      <c r="H54" s="5" t="inlineStr"/>
       <c r="I54" s="5" t="inlineStr"/>
       <c r="J54" s="5" t="inlineStr">
         <is>
-          <t>Flag for placebo subjects who crossed over at Week 16 and were re-randomized. Set to 'Y' if subject was originally randomized to placebo (TRT01P='Placebo') and has a DS record for crossover/re-randomization at Week 16. Used in T-14-1-1.</t>
+          <t>Stratification factor 1: baseline vIGA-AD severity (3 vs 4). Derived from randomization strata records or SUPPDM.QVAL where QNAM='VIGABASE' (or equivalent). Values: '3' (moderate) or '4' (severe). Used in CMH test for primary endpoint analysis (T-14-2-1).</t>
         </is>
       </c>
       <c r="K54" s="5" t="inlineStr">
         <is>
-          <t>Crossover flag set to 'Y' for placebo subjects re-randomized at Week 16 crossover point. Derived from DS domain records (DSDECOD indicating re-randomization) combined with original planned treatment being Placebo. Uses codelist NY.</t>
+          <t>Stratification factor 1 representing baseline vIGA-AD severity (3 or 4) from randomization strata. Derived from SUPPDM or randomization database. Uses sponsor-defined codelist ADSL_STRAT1.</t>
         </is>
       </c>
       <c r="L54" s="5" t="inlineStr">
@@ -6683,7 +6679,7 @@
       </c>
       <c r="M54" s="5" t="inlineStr">
         <is>
-          <t>DS domain variables (DSDECOD for crossover/re-randomization) not RAG-verified. Programmer must confirm DS domain coding for the Week 16 crossover event and re-randomization records.</t>
+          <t>SUPPDM variables not RAG-verified. Programmer must confirm the QNAM value used for baseline vIGA-AD in SUPPDM (e.g., QNAM='VIGABASE') or identify the randomization stratum dataset source.</t>
         </is>
       </c>
     </row>
@@ -6695,21 +6691,21 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>STRAT1</t>
+          <t>STRAT1N</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Stratification Factor 1</t>
+          <t>Stratification Factor 1 (N)</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="E55" s="5" t="n">
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
@@ -6725,12 +6721,12 @@
       <c r="I55" s="5" t="inlineStr"/>
       <c r="J55" s="5" t="inlineStr">
         <is>
-          <t>Stratification factor 1: baseline vIGA-AD severity (3 vs 4). Derived from randomization strata records or SUPPDM.QVAL where QNAM='VIGABASE' (or equivalent). Values: '3' (moderate) or '4' (severe). Used in CMH test for primary endpoint analysis (T-14-2-1).</t>
+          <t>Numeric code for STRAT1. 3=vIGA-AD score 3; 4=vIGA-AD score 4. See codelist ADSL_STRAT1N.</t>
         </is>
       </c>
       <c r="K55" s="5" t="inlineStr">
         <is>
-          <t>Stratification factor 1 representing baseline vIGA-AD severity (3 or 4) from randomization strata. Derived from SUPPDM or randomization database. Uses sponsor-defined codelist ADSL_STRAT1.</t>
+          <t>Numeric representation of STRAT1 for sorting. 3=Baseline vIGA-AD score 3; 4=Baseline vIGA-AD score 4. Uses sponsor-defined codelist ADSL_STRAT1N.</t>
         </is>
       </c>
       <c r="L55" s="5" t="inlineStr">
@@ -6740,172 +6736,176 @@
       </c>
       <c r="M55" s="5" t="inlineStr">
         <is>
-          <t>SUPPDM variables not RAG-verified. Programmer must confirm the QNAM value used for baseline vIGA-AD in SUPPDM (e.g., QNAM='VIGABASE') or identify the randomization stratum dataset source.</t>
+          <t>Dependent on STRAT1 derivation which requires SUPPDM source confirmation. Numeric code assignment must be confirmed with sponsor.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="30" customHeight="1">
-      <c r="A56" s="5" t="inlineStr">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>ADSL</t>
         </is>
       </c>
-      <c r="B56" s="5" t="inlineStr">
-        <is>
-          <t>STRAT1N</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>Stratification Factor 1 (N)</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr">
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>STRAT2</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>Stratification Factor 2</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>Perm</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr"/>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
+          <t>DM.AGE</t>
+        </is>
+      </c>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>Stratification factor 2: age group (Adolescent vs Adult). Derived from DM.AGE: 'Adolescent' if AGE &lt; 18; 'Adult' if AGE &gt;= 18. Used in CMH test for primary endpoint analysis (T-14-2-1).</t>
+        </is>
+      </c>
+      <c r="K56" s="4" t="inlineStr">
+        <is>
+          <t>Stratification factor 2 representing age group derived from DM.AGE: 'Adolescent' if AGE&lt;18; 'Adult' if AGE&gt;=18. Used for CMH test stratification in efficacy analyses. Uses sponsor-defined codelist ADSL_STRAT2.</t>
+        </is>
+      </c>
+      <c r="L56" s="4" t="inlineStr"/>
+      <c r="M56" s="4" t="inlineStr"/>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>ADSL</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>STRAT2N</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Stratification Factor 2 (N)</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>integer</t>
         </is>
       </c>
-      <c r="E56" s="5" t="n">
+      <c r="E57" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="F56" s="5" t="inlineStr">
-        <is>
-          <t>Derived</t>
-        </is>
-      </c>
-      <c r="G56" s="5" t="inlineStr">
-        <is>
-          <t>Perm</t>
-        </is>
-      </c>
-      <c r="H56" s="5" t="inlineStr"/>
-      <c r="I56" s="5" t="inlineStr"/>
-      <c r="J56" s="5" t="inlineStr">
-        <is>
-          <t>Numeric code for STRAT1. 3=vIGA-AD score 3; 4=vIGA-AD score 4. See codelist ADSL_STRAT1N.</t>
-        </is>
-      </c>
-      <c r="K56" s="5" t="inlineStr">
-        <is>
-          <t>Numeric representation of STRAT1 for sorting. 3=Baseline vIGA-AD score 3; 4=Baseline vIGA-AD score 4. Uses sponsor-defined codelist ADSL_STRAT1N.</t>
-        </is>
-      </c>
-      <c r="L56" s="5" t="inlineStr">
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>Perm</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr"/>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>DM.AGE</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>Numeric code for STRAT2. 1=Adolescent (AGE &lt; 18); 2=Adult (AGE &gt;= 18). See codelist ADSL_STRAT2N.</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>Numeric representation of STRAT2 for sorting. 1=Adolescent (AGE&lt;18); 2=Adult (AGE&gt;=18). Uses sponsor-defined codelist ADSL_STRAT2N.</t>
+        </is>
+      </c>
+      <c r="L57" s="3" t="inlineStr"/>
+      <c r="M57" s="3" t="inlineStr"/>
+    </row>
+    <row r="58" ht="30" customHeight="1">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>ADSL</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>STRAT3</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Stratification Factor 3</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="n">
+        <v>50</v>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>Perm</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="inlineStr"/>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>DM.COUNTRY</t>
+        </is>
+      </c>
+      <c r="J58" s="5" t="inlineStr">
+        <is>
+          <t>Stratification factor 3: geographic region. Derived from DM.COUNTRY mapped to regions (e.g., North America, Europe, Asia-Pacific, Rest of World). Used in CMH test for primary endpoint analysis (T-14-2-1).</t>
+        </is>
+      </c>
+      <c r="K58" s="5" t="inlineStr">
+        <is>
+          <t>Stratification factor 3 representing geographic region derived from DM.COUNTRY mapping to study-defined regions. Used for CMH test stratification in efficacy analyses. Uses sponsor-defined codelist ADSL_STRAT3.</t>
+        </is>
+      </c>
+      <c r="L58" s="5" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="M56" s="5" t="inlineStr">
-        <is>
-          <t>Dependent on STRAT1 derivation which requires SUPPDM source confirmation. Numeric code assignment must be confirmed with sponsor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="30" customHeight="1">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>ADSL</t>
-        </is>
-      </c>
-      <c r="B57" s="4" t="inlineStr">
-        <is>
-          <t>STRAT2</t>
-        </is>
-      </c>
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>Stratification Factor 2</t>
-        </is>
-      </c>
-      <c r="D57" s="4" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="E57" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>Derived</t>
-        </is>
-      </c>
-      <c r="G57" s="4" t="inlineStr">
-        <is>
-          <t>Perm</t>
-        </is>
-      </c>
-      <c r="H57" s="4" t="inlineStr"/>
-      <c r="I57" s="4" t="inlineStr">
-        <is>
-          <t>DM.AGE</t>
-        </is>
-      </c>
-      <c r="J57" s="4" t="inlineStr">
-        <is>
-          <t>Stratification factor 2: age group (Adolescent vs Adult). Derived from DM.AGE: 'Adolescent' if AGE &lt; 18; 'Adult' if AGE &gt;= 18. Used in CMH test for primary endpoint analysis (T-14-2-1).</t>
-        </is>
-      </c>
-      <c r="K57" s="4" t="inlineStr">
-        <is>
-          <t>Stratification factor 2 representing age group derived from DM.AGE: 'Adolescent' if AGE&lt;18; 'Adult' if AGE&gt;=18. Used for CMH test stratification in efficacy analyses. Uses sponsor-defined codelist ADSL_STRAT2.</t>
-        </is>
-      </c>
-      <c r="L57" s="4" t="inlineStr"/>
-      <c r="M57" s="4" t="inlineStr"/>
-    </row>
-    <row r="58" ht="30" customHeight="1">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>ADSL</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="inlineStr">
-        <is>
-          <t>STRAT2N</t>
-        </is>
-      </c>
-      <c r="C58" s="3" t="inlineStr">
-        <is>
-          <t>Stratification Factor 2 (N)</t>
-        </is>
-      </c>
-      <c r="D58" s="3" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="E58" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="F58" s="3" t="inlineStr">
-        <is>
-          <t>Derived</t>
-        </is>
-      </c>
-      <c r="G58" s="3" t="inlineStr">
-        <is>
-          <t>Perm</t>
-        </is>
-      </c>
-      <c r="H58" s="3" t="inlineStr"/>
-      <c r="I58" s="3" t="inlineStr">
-        <is>
-          <t>DM.AGE</t>
-        </is>
-      </c>
-      <c r="J58" s="3" t="inlineStr">
-        <is>
-          <t>Numeric code for STRAT2. 1=Adolescent (AGE &lt; 18); 2=Adult (AGE &gt;= 18). See codelist ADSL_STRAT2N.</t>
-        </is>
-      </c>
-      <c r="K58" s="3" t="inlineStr">
-        <is>
-          <t>Numeric representation of STRAT2 for sorting. 1=Adolescent (AGE&lt;18); 2=Adult (AGE&gt;=18). Uses sponsor-defined codelist ADSL_STRAT2N.</t>
-        </is>
-      </c>
-      <c r="L58" s="3" t="inlineStr"/>
-      <c r="M58" s="3" t="inlineStr"/>
+      <c r="M58" s="5" t="inlineStr">
+        <is>
+          <t>Region grouping algorithm from DM.COUNTRY must be confirmed with sponsor. Randomization stratum for region may differ from post-hoc grouping; programmer should check if region stratum is stored in SUPPDM.</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="5" t="inlineStr">
@@ -6915,21 +6915,21 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>STRAT3</t>
+          <t>STRAT3N</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Stratification Factor 3</t>
+          <t>Stratification Factor 3 (N)</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="E59" s="5" t="n">
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
@@ -6949,12 +6949,12 @@
       </c>
       <c r="J59" s="5" t="inlineStr">
         <is>
-          <t>Stratification factor 3: geographic region. Derived from DM.COUNTRY mapped to regions (e.g., North America, Europe, Asia-Pacific, Rest of World). Used in CMH test for primary endpoint analysis (T-14-2-1).</t>
+          <t>Numeric code for STRAT3. Numeric mapping of geographic region. See codelist ADSL_STRAT3N.</t>
         </is>
       </c>
       <c r="K59" s="5" t="inlineStr">
         <is>
-          <t>Stratification factor 3 representing geographic region derived from DM.COUNTRY mapping to study-defined regions. Used for CMH test stratification in efficacy analyses. Uses sponsor-defined codelist ADSL_STRAT3.</t>
+          <t>Numeric representation of STRAT3 (geographic region) for sorting. Uses sponsor-defined codelist ADSL_STRAT3N.</t>
         </is>
       </c>
       <c r="L59" s="5" t="inlineStr">
@@ -6964,7 +6964,7 @@
       </c>
       <c r="M59" s="5" t="inlineStr">
         <is>
-          <t>Region grouping algorithm from DM.COUNTRY must be confirmed with sponsor. Randomization stratum for region may differ from post-hoc grouping; programmer should check if region stratum is stored in SUPPDM.</t>
+          <t>Dependent on STRAT3 region grouping algorithm which must be confirmed with sponsor.</t>
         </is>
       </c>
     </row>
@@ -6976,21 +6976,21 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>STRAT3N</t>
+          <t>REGION1</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Stratification Factor 3 (N)</t>
+          <t>Geographic Region 1</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>text</t>
         </is>
       </c>
       <c r="E60" s="5" t="n">
-        <v>8</v>
+        <v>50</v>
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
@@ -7010,12 +7010,12 @@
       </c>
       <c r="J60" s="5" t="inlineStr">
         <is>
-          <t>Numeric code for STRAT3. Numeric mapping of geographic region. See codelist ADSL_STRAT3N.</t>
+          <t>Geographic region derived from DM.COUNTRY. Countries mapped to regions (e.g., 'North America', 'Europe', 'Asia-Pacific', 'Rest of World'). Used in demographic tables (T-14-1-2) and CMH stratification.</t>
         </is>
       </c>
       <c r="K60" s="5" t="inlineStr">
         <is>
-          <t>Numeric representation of STRAT3 (geographic region) for sorting. Uses sponsor-defined codelist ADSL_STRAT3N.</t>
+          <t>Geographic region derived from DM.COUNTRY using sponsor-defined country-to-region mapping. Uses sponsor-defined codelist ADSL_REGION1.</t>
         </is>
       </c>
       <c r="L60" s="5" t="inlineStr">
@@ -7025,7 +7025,7 @@
       </c>
       <c r="M60" s="5" t="inlineStr">
         <is>
-          <t>Dependent on STRAT3 region grouping algorithm which must be confirmed with sponsor.</t>
+          <t>Country-to-region mapping algorithm must be confirmed with sponsor. The exact region groupings need to be defined in the SAP or programming specifications.</t>
         </is>
       </c>
     </row>
@@ -7037,21 +7037,21 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>REGION1</t>
+          <t>REGION1N</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Geographic Region 1</t>
+          <t>Geographic Region 1 (N)</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="E61" s="5" t="n">
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
@@ -7071,12 +7071,12 @@
       </c>
       <c r="J61" s="5" t="inlineStr">
         <is>
-          <t>Geographic region derived from DM.COUNTRY. Countries mapped to regions (e.g., 'North America', 'Europe', 'Asia-Pacific', 'Rest of World'). Used in demographic tables (T-14-1-2) and CMH stratification.</t>
+          <t>Numeric code for REGION1. Numeric representation of geographic region for sorting. See codelist ADSL_REGION1N.</t>
         </is>
       </c>
       <c r="K61" s="5" t="inlineStr">
         <is>
-          <t>Geographic region derived from DM.COUNTRY using sponsor-defined country-to-region mapping. Uses sponsor-defined codelist ADSL_REGION1.</t>
+          <t>Numeric representation of REGION1 for sorting. Uses sponsor-defined codelist ADSL_REGION1N.</t>
         </is>
       </c>
       <c r="L61" s="5" t="inlineStr">
@@ -7086,404 +7086,398 @@
       </c>
       <c r="M61" s="5" t="inlineStr">
         <is>
-          <t>Country-to-region mapping algorithm must be confirmed with sponsor. The exact region groupings need to be defined in the SAP or programming specifications.</t>
+          <t>Dependent on REGION1 mapping algorithm which must be confirmed with sponsor.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="30" customHeight="1">
-      <c r="A62" s="5" t="inlineStr">
+      <c r="A62" s="4" t="inlineStr">
         <is>
           <t>ADSL</t>
         </is>
       </c>
-      <c r="B62" s="5" t="inlineStr">
-        <is>
-          <t>REGION1N</t>
-        </is>
-      </c>
-      <c r="C62" s="5" t="inlineStr">
-        <is>
-          <t>Geographic Region 1 (N)</t>
-        </is>
-      </c>
-      <c r="D62" s="5" t="inlineStr">
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>BRTHDTC</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>Date/Time of Birth</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>Predecessor</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>Perm</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="inlineStr"/>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t>DM.BRTHDTC</t>
+        </is>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t>Copied directly from DM.BRTHDTC. ISO 8601 date/time of birth.</t>
+        </is>
+      </c>
+      <c r="K62" s="4" t="inlineStr">
+        <is>
+          <t>Date/time of birth copied from DM.BRTHDTC in ISO 8601 format.</t>
+        </is>
+      </c>
+      <c r="L62" s="4" t="inlineStr"/>
+      <c r="M62" s="4" t="inlineStr"/>
+    </row>
+    <row r="63" ht="30" customHeight="1">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>ADSL</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>ARMNRS</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>Reason Arm Not Assigned</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>Predecessor</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>Perm</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>ADSL_ARMNRS</t>
+        </is>
+      </c>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>DM.ARMNRS</t>
+        </is>
+      </c>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>Copied directly from DM.ARMNRS. Describes the reason a subject was not assigned to an arm (e.g., screen failure).</t>
+        </is>
+      </c>
+      <c r="K63" s="3" t="inlineStr">
+        <is>
+          <t>Reason arm not assigned copied from DM.ARMNRS. Populated for subjects with missing ARMCD.</t>
+        </is>
+      </c>
+      <c r="L63" s="3" t="inlineStr"/>
+      <c r="M63" s="3" t="inlineStr"/>
+    </row>
+    <row r="64" ht="30" customHeight="1">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>ADSL</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>ACTARMUD</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>Description of Unplanned Actual Arm</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>Predecessor</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="inlineStr">
+        <is>
+          <t>Perm</t>
+        </is>
+      </c>
+      <c r="H64" s="4" t="inlineStr"/>
+      <c r="I64" s="4" t="inlineStr">
+        <is>
+          <t>DM.ACTARMUD</t>
+        </is>
+      </c>
+      <c r="J64" s="4" t="inlineStr">
+        <is>
+          <t>Copied directly from DM.ACTARMUD. Describes the actual arm if it was unplanned.</t>
+        </is>
+      </c>
+      <c r="K64" s="4" t="inlineStr">
+        <is>
+          <t>Description of unplanned actual arm copied from DM.ACTARMUD.</t>
+        </is>
+      </c>
+      <c r="L64" s="4" t="inlineStr"/>
+      <c r="M64" s="4" t="inlineStr"/>
+    </row>
+    <row r="65" ht="30" customHeight="1">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>ADSL</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>AGEUN</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>Age Units (N)</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
         <is>
           <t>integer</t>
         </is>
       </c>
-      <c r="E62" s="5" t="n">
+      <c r="E65" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="F62" s="5" t="inlineStr">
-        <is>
-          <t>Derived</t>
-        </is>
-      </c>
-      <c r="G62" s="5" t="inlineStr">
-        <is>
-          <t>Perm</t>
-        </is>
-      </c>
-      <c r="H62" s="5" t="inlineStr"/>
-      <c r="I62" s="5" t="inlineStr">
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>ADSL_AGEUN</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>DM.AGEU</t>
+        </is>
+      </c>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>Numeric code for AGEU. See codelist ADSL_AGEUN.</t>
+        </is>
+      </c>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>Numeric version of AGEU. Assigned from ADSL_AGEUN codelist numeric decode.</t>
+        </is>
+      </c>
+      <c r="L65" s="3" t="inlineStr"/>
+      <c r="M65" s="3" t="inlineStr"/>
+    </row>
+    <row r="66" ht="30" customHeight="1">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>ADSL</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>COUNTRYN</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Country (N)</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>Perm</t>
+        </is>
+      </c>
+      <c r="H66" s="4" t="inlineStr">
+        <is>
+          <t>COUNTRYN</t>
+        </is>
+      </c>
+      <c r="I66" s="4" t="inlineStr">
         <is>
           <t>DM.COUNTRY</t>
         </is>
       </c>
-      <c r="J62" s="5" t="inlineStr">
-        <is>
-          <t>Numeric code for REGION1. Numeric representation of geographic region for sorting. See codelist ADSL_REGION1N.</t>
-        </is>
-      </c>
-      <c r="K62" s="5" t="inlineStr">
-        <is>
-          <t>Numeric representation of REGION1 for sorting. Uses sponsor-defined codelist ADSL_REGION1N.</t>
-        </is>
-      </c>
-      <c r="L62" s="5" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="M62" s="5" t="inlineStr">
-        <is>
-          <t>Dependent on REGION1 mapping algorithm which must be confirmed with sponsor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="30" customHeight="1">
-      <c r="A63" s="4" t="inlineStr">
+      <c r="J66" s="4" t="inlineStr">
+        <is>
+          <t>Numeric code for COUNTRY. See codelist COUNTRYN.</t>
+        </is>
+      </c>
+      <c r="K66" s="4" t="inlineStr">
+        <is>
+          <t>Numeric version of COUNTRY. Assigned from COUNTRYN codelist numeric decode.</t>
+        </is>
+      </c>
+      <c r="L66" s="4" t="inlineStr"/>
+      <c r="M66" s="4" t="inlineStr"/>
+    </row>
+    <row r="67" ht="30" customHeight="1">
+      <c r="A67" s="3" t="inlineStr">
         <is>
           <t>ADSL</t>
         </is>
       </c>
-      <c r="B63" s="4" t="inlineStr">
-        <is>
-          <t>BRTHDTC</t>
-        </is>
-      </c>
-      <c r="C63" s="4" t="inlineStr">
-        <is>
-          <t>Date/Time of Birth</t>
-        </is>
-      </c>
-      <c r="D63" s="4" t="inlineStr">
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>ARMNRSN</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>Reason Arm Not Assigned (N)</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>integer</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>Perm</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>ADSL_ARMNRSN</t>
+        </is>
+      </c>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>DM.ARMNRS</t>
+        </is>
+      </c>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>Numeric code for ARMNRS. See codelist ADSL_ARMNRSN.</t>
+        </is>
+      </c>
+      <c r="K67" s="3" t="inlineStr">
+        <is>
+          <t>Numeric version of ARMNRS. Assigned from ADSL_ARMNRSN codelist numeric decode.</t>
+        </is>
+      </c>
+      <c r="L67" s="3" t="inlineStr"/>
+      <c r="M67" s="3" t="inlineStr"/>
+    </row>
+    <row r="68" ht="30" customHeight="1">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>ADSL</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>REGION</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Geographic Region</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="E63" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F63" s="4" t="inlineStr">
-        <is>
-          <t>Predecessor</t>
-        </is>
-      </c>
-      <c r="G63" s="4" t="inlineStr">
-        <is>
-          <t>Perm</t>
-        </is>
-      </c>
-      <c r="H63" s="4" t="inlineStr"/>
-      <c r="I63" s="4" t="inlineStr">
-        <is>
-          <t>DM.BRTHDTC</t>
-        </is>
-      </c>
-      <c r="J63" s="4" t="inlineStr">
-        <is>
-          <t>Copied directly from DM.BRTHDTC. ISO 8601 date/time of birth.</t>
-        </is>
-      </c>
-      <c r="K63" s="4" t="inlineStr">
-        <is>
-          <t>Date/time of birth copied from DM.BRTHDTC in ISO 8601 format.</t>
-        </is>
-      </c>
-      <c r="L63" s="4" t="inlineStr"/>
-      <c r="M63" s="4" t="inlineStr"/>
-    </row>
-    <row r="64" ht="30" customHeight="1">
-      <c r="A64" s="3" t="inlineStr">
-        <is>
-          <t>ADSL</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>ARMNRS</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="inlineStr">
-        <is>
-          <t>Reason Arm Not Assigned</t>
-        </is>
-      </c>
-      <c r="D64" s="3" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="E64" s="3" t="n">
-        <v>200</v>
-      </c>
-      <c r="F64" s="3" t="inlineStr">
-        <is>
-          <t>Predecessor</t>
-        </is>
-      </c>
-      <c r="G64" s="3" t="inlineStr">
-        <is>
-          <t>Perm</t>
-        </is>
-      </c>
-      <c r="H64" s="3" t="inlineStr">
-        <is>
-          <t>ADSL_ARMNRS</t>
-        </is>
-      </c>
-      <c r="I64" s="3" t="inlineStr">
-        <is>
-          <t>DM.ARMNRS</t>
-        </is>
-      </c>
-      <c r="J64" s="3" t="inlineStr">
-        <is>
-          <t>Copied directly from DM.ARMNRS. Describes the reason a subject was not assigned to an arm (e.g., screen failure).</t>
-        </is>
-      </c>
-      <c r="K64" s="3" t="inlineStr">
-        <is>
-          <t>Reason arm not assigned copied from DM.ARMNRS. Populated for subjects with missing ARMCD.</t>
-        </is>
-      </c>
-      <c r="L64" s="3" t="inlineStr"/>
-      <c r="M64" s="3" t="inlineStr"/>
-    </row>
-    <row r="65" ht="30" customHeight="1">
-      <c r="A65" s="4" t="inlineStr">
-        <is>
-          <t>ADSL</t>
-        </is>
-      </c>
-      <c r="B65" s="4" t="inlineStr">
-        <is>
-          <t>ACTARMUD</t>
-        </is>
-      </c>
-      <c r="C65" s="4" t="inlineStr">
-        <is>
-          <t>Description of Unplanned Actual Arm</t>
-        </is>
-      </c>
-      <c r="D65" s="4" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="E65" s="4" t="n">
-        <v>200</v>
-      </c>
-      <c r="F65" s="4" t="inlineStr">
-        <is>
-          <t>Predecessor</t>
-        </is>
-      </c>
-      <c r="G65" s="4" t="inlineStr">
-        <is>
-          <t>Perm</t>
-        </is>
-      </c>
-      <c r="H65" s="4" t="inlineStr"/>
-      <c r="I65" s="4" t="inlineStr">
-        <is>
-          <t>DM.ACTARMUD</t>
-        </is>
-      </c>
-      <c r="J65" s="4" t="inlineStr">
-        <is>
-          <t>Copied directly from DM.ACTARMUD. Describes the actual arm if it was unplanned.</t>
-        </is>
-      </c>
-      <c r="K65" s="4" t="inlineStr">
-        <is>
-          <t>Description of unplanned actual arm copied from DM.ACTARMUD.</t>
-        </is>
-      </c>
-      <c r="L65" s="4" t="inlineStr"/>
-      <c r="M65" s="4" t="inlineStr"/>
-    </row>
-    <row r="66" ht="30" customHeight="1">
-      <c r="A66" s="3" t="inlineStr">
-        <is>
-          <t>ADSL</t>
-        </is>
-      </c>
-      <c r="B66" s="3" t="inlineStr">
-        <is>
-          <t>AGEUN</t>
-        </is>
-      </c>
-      <c r="C66" s="3" t="inlineStr">
-        <is>
-          <t>Age Units (N)</t>
-        </is>
-      </c>
-      <c r="D66" s="3" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="E66" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="F66" s="3" t="inlineStr">
-        <is>
-          <t>Derived</t>
-        </is>
-      </c>
-      <c r="G66" s="3" t="inlineStr">
-        <is>
-          <t>Req</t>
-        </is>
-      </c>
-      <c r="H66" s="3" t="inlineStr">
-        <is>
-          <t>ADSL_AGEUN</t>
-        </is>
-      </c>
-      <c r="I66" s="3" t="inlineStr">
-        <is>
-          <t>DM.AGEU</t>
-        </is>
-      </c>
-      <c r="J66" s="3" t="inlineStr">
-        <is>
-          <t>Numeric code for AGEU. See codelist ADSL_AGEUN.</t>
-        </is>
-      </c>
-      <c r="K66" s="3" t="inlineStr">
-        <is>
-          <t>Numeric version of AGEU. Assigned from ADSL_AGEUN codelist numeric decode.</t>
-        </is>
-      </c>
-      <c r="L66" s="3" t="inlineStr"/>
-      <c r="M66" s="3" t="inlineStr"/>
-    </row>
-    <row r="67" ht="30" customHeight="1">
-      <c r="A67" s="4" t="inlineStr">
-        <is>
-          <t>ADSL</t>
-        </is>
-      </c>
-      <c r="B67" s="4" t="inlineStr">
-        <is>
-          <t>COUNTRYN</t>
-        </is>
-      </c>
-      <c r="C67" s="4" t="inlineStr">
-        <is>
-          <t>Country (N)</t>
-        </is>
-      </c>
-      <c r="D67" s="4" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="E67" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="F67" s="4" t="inlineStr">
-        <is>
-          <t>Derived</t>
-        </is>
-      </c>
-      <c r="G67" s="4" t="inlineStr">
-        <is>
-          <t>Perm</t>
-        </is>
-      </c>
-      <c r="H67" s="4" t="inlineStr">
-        <is>
-          <t>COUNTRYN</t>
-        </is>
-      </c>
-      <c r="I67" s="4" t="inlineStr">
-        <is>
-          <t>DM.COUNTRY</t>
-        </is>
-      </c>
-      <c r="J67" s="4" t="inlineStr">
-        <is>
-          <t>Numeric code for COUNTRY. See codelist COUNTRYN.</t>
-        </is>
-      </c>
-      <c r="K67" s="4" t="inlineStr">
-        <is>
-          <t>Numeric version of COUNTRY. Assigned from COUNTRYN codelist numeric decode.</t>
-        </is>
-      </c>
-      <c r="L67" s="4" t="inlineStr"/>
-      <c r="M67" s="4" t="inlineStr"/>
-    </row>
-    <row r="68" ht="30" customHeight="1">
-      <c r="A68" s="3" t="inlineStr">
-        <is>
-          <t>ADSL</t>
-        </is>
-      </c>
-      <c r="B68" s="3" t="inlineStr">
-        <is>
-          <t>ARMNRSN</t>
-        </is>
-      </c>
-      <c r="C68" s="3" t="inlineStr">
-        <is>
-          <t>Reason Arm Not Assigned (N)</t>
-        </is>
-      </c>
-      <c r="D68" s="3" t="inlineStr">
-        <is>
-          <t>integer</t>
-        </is>
-      </c>
-      <c r="E68" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="F68" s="3" t="inlineStr">
-        <is>
-          <t>Derived</t>
-        </is>
-      </c>
-      <c r="G68" s="3" t="inlineStr">
-        <is>
-          <t>Perm</t>
-        </is>
-      </c>
-      <c r="H68" s="3" t="inlineStr">
-        <is>
-          <t>ADSL_ARMNRSN</t>
-        </is>
-      </c>
-      <c r="I68" s="3" t="inlineStr">
-        <is>
-          <t>DM.ARMNRS</t>
-        </is>
-      </c>
-      <c r="J68" s="3" t="inlineStr">
-        <is>
-          <t>Numeric code for ARMNRS. See codelist ADSL_ARMNRSN.</t>
-        </is>
-      </c>
-      <c r="K68" s="3" t="inlineStr">
-        <is>
-          <t>Numeric version of ARMNRS. Assigned from ADSL_ARMNRSN codelist numeric decode.</t>
-        </is>
-      </c>
-      <c r="L68" s="3" t="inlineStr"/>
-      <c r="M68" s="3" t="inlineStr"/>
+      <c r="E68" t="n">
+        <v>40</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Perm</t>
+        </is>
+      </c>
+      <c r="H68" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="I68" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Simulated for the APX-DRM-301 training example.</t>
+        </is>
+      </c>
+      <c r="K68" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="L68" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="M68" t="e">
+        <v>#N/A</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -7493,12 +7487,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>REGION</t>
+          <t>DCSREASN</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Geographic Region</t>
+          <t>Discontinuation Reason</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -7548,21 +7542,21 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>DCSREASN</t>
+          <t>WEIGHT</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Discontinuation Reason</t>
+          <t>Body Weight (kg)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>float</t>
         </is>
       </c>
       <c r="E70" t="n">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -7603,12 +7597,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>WEIGHT</t>
+          <t>BMI</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Body Weight (kg)</t>
+          <t>Body Mass Index (kg/m2)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -7658,17 +7652,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>BMI</t>
+          <t>EASIBL</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Body Mass Index (kg/m2)</t>
+          <t>Baseline EASI Total Score</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="E72" t="n">
@@ -7713,21 +7707,21 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>EASIBL</t>
+          <t>EASIBLC</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Baseline EASI Total Score</t>
+          <t>Baseline EASI Severity Category</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>text</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -7768,12 +7762,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>EASIBLC</t>
+          <t>IGABLC</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Baseline EASI Severity Category</t>
+          <t>Baseline vIGA-AD Category</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -7823,21 +7817,21 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>IGABLC</t>
+          <t>BSABL</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Baseline vIGA-AD Category</t>
+          <t>Baseline % BSA Affected</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>float</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -7878,17 +7872,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>BSABL</t>
+          <t>WPNRSBL</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Baseline % BSA Affected</t>
+          <t>Baseline WP-NRS Score</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="E76" t="n">
@@ -7933,12 +7927,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>WPNRSBL</t>
+          <t>POEMBL</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Baseline WP-NRS Score</t>
+          <t>Baseline POEM Total Score</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -7988,12 +7982,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>POEMBL</t>
+          <t>DLQIBL</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Baseline POEM Total Score</t>
+          <t>Baseline DLQI/CDLQI Total Score</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -8043,17 +8037,17 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>DLQIBL</t>
+          <t>ADDUR</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Baseline DLQI/CDLQI Total Score</t>
+          <t>Duration of Atopic Dermatitis (years)</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>float</t>
         </is>
       </c>
       <c r="E79" t="n">
@@ -8098,21 +8092,21 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>ADDUR</t>
+          <t>ATOPCMB</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Duration of Atopic Dermatitis (years)</t>
+          <t>Atopic Comorbidities Present</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>text</t>
         </is>
       </c>
       <c r="E80" t="n">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -8153,12 +8147,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>ATOPCMB</t>
+          <t>PRSYSTAD</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Atopic Comorbidities Present</t>
+          <t>Prior Systemic Therapy for AD</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -8197,61 +8191,6 @@
         <v>#N/A</v>
       </c>
       <c r="M81" t="e">
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>ADSL</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>PRSYSTAD</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>Prior Systemic Therapy for AD</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="E82" t="n">
-        <v>40</v>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>Derived</t>
-        </is>
-      </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>Perm</t>
-        </is>
-      </c>
-      <c r="H82" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="I82" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="J82" t="inlineStr">
-        <is>
-          <t>Simulated for the APX-DRM-301 training example.</t>
-        </is>
-      </c>
-      <c r="K82" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="L82" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="M82" t="e">
         <v>#N/A</v>
       </c>
     </row>

</xml_diff>